<commit_message>
Risk analysis update and report
</commit_message>
<xml_diff>
--- a/1.Planning Documents/CW Risks.xlsx
+++ b/1.Planning Documents/CW Risks.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10209"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10329"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/stuartbaker/Documents/GitHub/Software-Engineering-Project/Plan/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/stuartbaker/Documents/GitHub/Software-Engineering-Project/1.Planning Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7137E90-030E-B741-A075-E59D5ABC3982}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CE50FCC-59E5-E24A-A33E-AA6C67620251}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="380" yWindow="500" windowWidth="28040" windowHeight="15980" xr2:uid="{96C42A70-5923-F145-81DA-CC33F505D3E0}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="59">
   <si>
     <t>Affects</t>
   </si>
@@ -179,9 +179,6 @@
     <t>Poor communication (medium); luck (high); cold weather (high)</t>
   </si>
   <si>
-    <t>Communincate when unwell and its affect on performance; change meetings and wokrload to accommodate</t>
-  </si>
-  <si>
     <t>Traffic, trains and buses</t>
   </si>
   <si>
@@ -198,6 +195,24 @@
   </si>
   <si>
     <t>Missing uni; missing meetings; lowers morale; lateness</t>
+  </si>
+  <si>
+    <t>Other coursework</t>
+  </si>
+  <si>
+    <t>Less time for this project; fall behind schedule; stress</t>
+  </si>
+  <si>
+    <t>Alert teammates if other coursework is time consuming; share workload; be flexible with schedule</t>
+  </si>
+  <si>
+    <t>Poor communication (medium); time management (high); stress from worklaod (low)</t>
+  </si>
+  <si>
+    <t>Communincate when unwell and its affect on performance; change meetings and workload to accommodate</t>
+  </si>
+  <si>
+    <t>Inform teammates of any struggles or priorities; allow flexibility for catchup time; keep up  with meetings/decisions</t>
   </si>
 </sst>
 </file>
@@ -626,7 +641,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4FF717A5-D0E1-0E43-BC29-58ACCCC5A807}">
-  <dimension ref="B2:F12"/>
+  <dimension ref="B2:F13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="6" width="40.83203125" customWidth="1"/>
@@ -790,7 +805,7 @@
         <v>44</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D11" s="3" t="s">
         <v>45</v>
@@ -799,24 +814,41 @@
         <v>46</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
     </row>
     <row r="12" spans="2:6" ht="40" x14ac:dyDescent="0.2">
       <c r="B12" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C12" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="13" spans="2:6" ht="60" x14ac:dyDescent="0.2">
+      <c r="B13" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="D12" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="F12" s="4" t="s">
-        <v>52</v>
+      <c r="C13" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>